<commit_message>
Automobile model was added
</commit_message>
<xml_diff>
--- a/НИРС2/hCVT model/CVT.xlsx
+++ b/НИРС2/hCVT model/CVT.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Баунти\Diplom\НИРС2\hCVT model\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45359568-32AE-4AC8-A29C-5AA65B9AFA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE7F288-C8A4-407A-9202-586E6813AF7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,10 +31,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>